<commit_message>
feat: balances, locations, usages de location et migrations Prisma
Ajoute les modules balances (lignes, import Excel), rentals et rental-usages, les migrations associées, le schéma Swagger d'enveloppe API, et met à jour Postman, les clients/tiers et les tests e2e. Harmonise les imports nommés sur une seule ligne là où ils étaient multi-lignes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/assets/xlsx/employe-import-template.xlsx
+++ b/src/assets/xlsx/employe-import-template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\compta-api\src\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6C495B3-3489-414F-9C8E-AB61A1E6B8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFDB3DB-6FAF-4B0E-AB1B-9CF1EE2BD18D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40485" yWindow="2280" windowWidth="21600" windowHeight="11295" xr2:uid="{1AC49CE9-6B7F-48F0-8745-27FF65013EB6}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{1AC49CE9-6B7F-48F0-8745-27FF65013EB6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Importation Employé" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>